<commit_message>
docs(FCC-core): add Claude-response column to high-level design (answers to user's 3 data-layer review comments)
Preserved the user's comments; added a 'Claude response' column on the Overview, Connect-
accounts, and Income+spending rows: account types (banking/investments/retirement/credit/
loans + manual), connect-once -> auto daily+on-open refresh (Plaid, read-only, privacy
spike flagged), progressive-connect onboarding for hesitant users, and the overview-objective
gap (fix in v1.1). Design content unchanged (still v1.0); v1.1 carries the 4 changes.
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/FCC-core-highlevel-design-v1.0-2026-06-30.xlsx
+++ b/docs/FCC-core-55-70/FCC-core-highlevel-design-v1.0-2026-06-30.xlsx
@@ -2,9 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="33600" windowHeight="19880" tabRatio="600" firstSheet="0" activeTab="4" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Overview &amp; principles" sheetId="1" state="visible" r:id="rId1"/>
@@ -14,14 +13,14 @@
     <sheet name="Journeys" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,19 +29,30 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Courier New"/>
+      <family val="1"/>
+      <sz val="9"/>
+    </font>
+    <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
-    <font>
-      <b val="1"/>
-    </font>
-    <font>
-      <name val="Courier New"/>
-      <sz val="9"/>
-    </font>
   </fonts>
-  <fills count="6">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -51,17 +61,27 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001A1A18"/>
+        <fgColor rgb="FF1A1A18"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
+        <fgColor rgb="FFFFF2CC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF7E6"/>
+        <fgColor rgb="FFFFF7E6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001A1A18"/>
       </patternFill>
     </fill>
     <fill>
@@ -70,12 +90,27 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD9D9D9"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD9D9D9"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -96,7 +131,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -122,9 +157,15 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -487,13 +528,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:E12"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="96" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="49.33203125" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -517,8 +559,13 @@
           <t>💬 Your comments</t>
         </is>
       </c>
-    </row>
-    <row r="2" ht="150" customHeight="1">
+      <c r="E1" s="9" t="inlineStr">
+        <is>
+          <t>💬 Claude response</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="220" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>OVERVIEW</t>
@@ -529,10 +576,21 @@
           <t>The 55-70 core is the shared front-door of FinWise for people in the hand-off zone between working and retired: the still-working 55-65 (top of the 36-65 working-years product) and the recently-retired 65-70 (front of the 65+ product). It is ONE product with two faces it flexes between. Underneath every screen sit three stacked layers: FOUNDATION (your real income, spending and connected accounts roll up into one true picture, with the timing of lumpy income and lumpy bills captured by month), the HERO/hook (for the still-working it is Grow and Track your investments; for the retired it is a Safe-to-spend-this-month paycheck number that genuinely rises and falls month to month), and REASSURANCE (the will-it-last / retirement-confidence answer, which lives in exactly one place and is the same number everywhere it appears). On top of all of it, FinWise acts as your CHIEF OF STAFF for the handful of big, mostly-irreversible decisions of this decade (when to claim Social Security, the retirement transition itself, required withdrawals): it lays out your real numbers, runs the options side-by-side in your own dollars, handles the deadlines and reminders, and shows the math of the best path under assumptions YOU set -- but it never tells you what to do and never claims to know the future. You always decide. The whole thing fits a phone, is written so a founder with zero finance background understands every word, and treats every number as sacred because one wrong number loses trust forever -- which is exactly why the retired Safe-to-spend hero is built as a real new month-by-month engine, not faked from a yearly average.</t>
         </is>
       </c>
-      <c r="C2" s="4" t="inlineStr"/>
-      <c r="D2" s="4" t="inlineStr"/>
-    </row>
-    <row r="3">
+      <c r="C2" s="4" t="n"/>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>Foundation layer only shows income, spending, and connected accounts as true picture. Three questions (1) Are these connected accounts checking, savings, investments, credit card or something different? (2) Via Plaid or anyother third party tool can the app actually pull real data without prompted by user daily? How will data be pulled, and at what frequency? (3) We said for this group - FinWise gives 36-to-65-year-olds one honest, engaging place to see their whole financial picture — led by how their investments and net worth are actually growing — and to explore the consequences of their big money choices for themselves. It matters because this group has the most money and the most at stake, yet no app shows them the whole truth clearly AND makes it something they actually want to open week to week. But that's not reflected in this overview or did I miss something?</t>
+        </is>
+      </c>
+      <c r="E2" s="10" t="inlineStr">
+        <is>
+          <t>(1) ACCOUNT TYPES: all of them — banking (checking/savings/cash management), INVESTMENTS (brokerage + retirement 401(k)/IRA — where the growth &amp; net-worth number lives), credit cards + loans; manual-add for what can't be linked (home value, pension, private assets).
+(2) PULL: yes, NO daily prompting. Connect each institution ONCE via an aggregator (Plaid is the standard); the connection persists. Data then auto-pulls — a DAILY refresh + a refresh each time the app opens. Read-only (we can never move money). ⚠ Privacy spike: Plaid routes data through its servers in transit, so 'never leaves your device' isn't literal — honest posture = read-only, on-device storage, encrypted, minimal retention, never sold (carries to the PRD/technical stage).
+(3) OBJECTIVE: you're right — it's a gap. The overview describes the shared core but doesn't foreground each group's objective/hook. FIX in v1.1: rewrite the overview to carry both groups' approved objectives (Grow &amp; Track / week-to-week for 55-65; safe-to-spend / worry-less for 65-70).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="48" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
         <is>
           <t>Principle 1</t>
@@ -543,10 +601,14 @@
           <t>Chief of staff, not advisor: we tee up the big decision (your numbers, the options, the trade-offs, the steps, the deadlines, and the best-math path under YOUR assumptions) -- you always decide. We never say 'do this' and never make a buy, sell, or claim recommendation.</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr"/>
-      <c r="D3" s="4" t="inlineStr"/>
-    </row>
-    <row r="4">
+      <c r="C3" s="4" t="n"/>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>Shall we also talk about - we surface right things at the right time - kind of what needs your attention.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="32" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
         <is>
           <t>Principle 2</t>
@@ -557,10 +619,10 @@
           <t>Never predict the future: we run scenarios for an honest, well-grounded estimate (a range of outcomes and the odds), never a single confident forecast. Every projected number is labeled an estimate, not a promise.</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr"/>
-      <c r="D4" s="4" t="inlineStr"/>
-    </row>
-    <row r="5">
+      <c r="C4" s="4" t="n"/>
+      <c r="D4" s="4" t="n"/>
+    </row>
+    <row r="5" ht="16" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
           <t>Principle 3</t>
@@ -571,10 +633,10 @@
           <t>Show what's true first: every screen rests on your real, connected numbers. The truth comes before the pep talk.</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr"/>
-      <c r="D5" s="4" t="inlineStr"/>
-    </row>
-    <row r="6">
+      <c r="C5" s="4" t="n"/>
+      <c r="D5" s="4" t="n"/>
+    </row>
+    <row r="6" ht="64" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
           <t>Principle 4</t>
@@ -585,10 +647,10 @@
           <t>Safe-to-spend is REAL month by month, never a flat yearly average: a retiree may get one big pension payment in March and a big property-tax bill in November -- spreading the year evenly would be a lie. Each month is computed from the actual timing of money coming in and the known big bills going out. This requires a new month-by-month engine; we build it rather than fake it.</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr"/>
-      <c r="D6" s="4" t="inlineStr"/>
-    </row>
-    <row r="7">
+      <c r="C6" s="4" t="n"/>
+      <c r="D6" s="4" t="n"/>
+    </row>
+    <row r="7" ht="48" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
           <t>Principle 5</t>
@@ -599,10 +661,10 @@
           <t>Month-by-month numeric accuracy is non-negotiable: one concept, one engine, one number, the same on every screen. A wrong number loses trust. The will-it-last odds in particular have ONE home and every other screen shows that same number.</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr"/>
-      <c r="D7" s="4" t="inlineStr"/>
-    </row>
-    <row r="8">
+      <c r="C7" s="4" t="n"/>
+      <c r="D7" s="4" t="n"/>
+    </row>
+    <row r="8" ht="64" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
         <is>
           <t>Principle 6</t>
@@ -613,10 +675,10 @@
           <t>Plain English, no jargon: every word readable by someone with no finance background; we say 'compared to the stock market' not 'benchmark', 'best-to-worst-case range' not 'percentile bands', 'too much in one stock' not 'concentration'. Acronyms are always spelled out (Social Security; required minimum withdrawal -- the amount the government makes you take out of pre-tax retirement accounts each year starting at 73; individual retirement account).</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr"/>
-      <c r="D8" s="4" t="inlineStr"/>
-    </row>
-    <row r="9">
+      <c r="C8" s="4" t="n"/>
+      <c r="D8" s="4" t="n"/>
+    </row>
+    <row r="9" ht="16" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
         <is>
           <t>Principle 7</t>
@@ -627,10 +689,10 @@
           <t>Mobile-first: everything fits and is readable on one phone screen; the hero number is glanceable in two seconds.</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr"/>
-      <c r="D9" s="4" t="inlineStr"/>
-    </row>
-    <row r="10">
+      <c r="C9" s="4" t="n"/>
+      <c r="D9" s="4" t="n"/>
+    </row>
+    <row r="10" ht="32" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
           <t>Principle 8</t>
@@ -641,10 +703,10 @@
           <t>Two lenses, one core: 'Grow and Track' for the still-working 55-65, 'Worry less, live more' / Safe-to-spend for the early-retired 65-70 -- the same foundation and engines, a different hero.</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr"/>
-      <c r="D10" s="4" t="inlineStr"/>
-    </row>
-    <row r="11">
+      <c r="C10" s="4" t="n"/>
+      <c r="D10" s="4" t="n"/>
+    </row>
+    <row r="11" ht="32" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
         <is>
           <t>Principle 9</t>
@@ -655,10 +717,10 @@
           <t>Pointed but warm voice: put a number on the truth, celebrate real wins, stay calm and steady for retirees. Never alarmist, never preachy.</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr"/>
-      <c r="D11" s="4" t="inlineStr"/>
-    </row>
-    <row r="12">
+      <c r="C11" s="4" t="n"/>
+      <c r="D11" s="4" t="n"/>
+    </row>
+    <row r="12" ht="32" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
         <is>
           <t>Principle 10</t>
@@ -669,8 +731,8 @@
           <t>Colorblind-safe and accessible: never rely on red/green alone -- pair color with a word, icon, or shape; readable type, large tap targets.</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr"/>
-      <c r="D12" s="4" t="inlineStr"/>
+      <c r="C12" s="4" t="n"/>
+      <c r="D12" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -683,8 +745,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:H11"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
     <col width="50" customWidth="1" min="2" max="2"/>
@@ -693,6 +755,7 @@
     <col width="34" customWidth="1" min="5" max="5"/>
     <col width="11" customWidth="1" min="6" max="6"/>
     <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -731,8 +794,13 @@
           <t>💬 Comments</t>
         </is>
       </c>
-    </row>
-    <row r="2">
+      <c r="H1" s="9" t="inlineStr">
+        <is>
+          <t>💬 Claude response</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="220" customHeight="1">
       <c r="A2" s="6" t="inlineStr">
         <is>
           <t>Connect accounts -&gt; whole-picture net worth</t>
@@ -758,10 +826,20 @@
           <t>Reuses the built net-worth math (src/domain/networth) and NetWorthScreen; the secure read-only sync seam is the one genuinely new connector piece.</t>
         </is>
       </c>
-      <c r="F2" s="4" t="inlineStr"/>
-      <c r="G2" s="4" t="inlineStr"/>
-    </row>
-    <row r="3">
+      <c r="F2" s="4" t="n"/>
+      <c r="G2" s="4" t="inlineStr">
+        <is>
+          <t>Is it one time pull, daily, or initiated by user? What if user is hesitant to connects account in the beginning?</t>
+        </is>
+      </c>
+      <c r="H2" s="10" t="inlineStr">
+        <is>
+          <t>One-time connect -&gt; AUTOMATIC refresh (daily + on-open), NOT user-initiated each day. Read-only.
+HESITANCY (we don't force it): (a) START WITHOUT CONNECTING — manual/partial entry so they see the first 'aha' (net worth / a rough safe-to-spend) before linking anything; (b) PROGRESSIVE CONNECT — link the ONE account that unlocks the hero they care about (brokerage -&gt; Grow &amp; Track; checking + income -&gt; safe-to-spend), then invite more; (c) lead with read-only / on-device / never-sold as the trust + the reward. v1.1 adds a progressive-connect onboarding path.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="220" customHeight="1">
       <c r="A3" s="6" t="inlineStr">
         <is>
           <t>Income + spending by month, including dated big bills and lumpy income</t>
@@ -787,10 +865,19 @@
           <t>Reuses cashflowYear (per-month inflow/outflow/net) + budget spendByMonth + income engine for the working-life inflows. NEW: a dated big-bill / lumpy-expense input that places named bills in their month (today the dated-bill path covers tuition/loans for a student persona only -- this extends it to retiree bills).</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr"/>
-      <c r="G3" s="4" t="inlineStr"/>
-    </row>
-    <row r="4">
+      <c r="F3" s="4" t="n"/>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>How all this information will be captured and at what frequency?</t>
+        </is>
+      </c>
+      <c r="H3" s="10" t="inlineStr">
+        <is>
+          <t>Mostly AUTOMATIC from the connected accounts on the same daily/on-open refresh (deposits -&gt; income, transactions -&gt; spending). DATED big bills (property tax in Nov, a pension lump in Dec) and anything not connected are MANUALLY added — that's what keeps safe-to-spend honest MONTH-BY-MONTH. So: auto from accounts + manual for dated lumpy items. v1.1 clarifies this on the row.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="208" customHeight="1">
       <c r="A4" s="6" t="inlineStr">
         <is>
           <t>Grow &amp; Track investments (the still-working hero)</t>
@@ -816,10 +903,14 @@
           <t>Reuses the Performance + portfolio-return engine (src/domain/performance: buildPerformance, attribution, market comparison, totalROI, portfolioTrend) and PerformanceScreen.</t>
         </is>
       </c>
-      <c r="F4" s="4" t="inlineStr"/>
-      <c r="G4" s="4" t="inlineStr"/>
-    </row>
-    <row r="5">
+      <c r="F4" s="4" t="n"/>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Does this also answer questions about Can I efford an home, or kids college, or take care of parents as we laid out in strategy doc - "Your chief of staff for the BUILDING years — guides you through your investments, the home, the kids' college, and the run-up to retirement, so you build the life you're working toward. 'Grow' = watch your money grow (the hook); 'Track' = always know you're on track.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="320" customHeight="1">
       <c r="A5" s="6" t="inlineStr">
         <is>
           <t>Safe-to-spend-in-retirement paycheck (the retired hero) -- NEW month-by-month engine</t>
@@ -845,10 +936,10 @@
           <t>NEW month-by-month retirement-income + safe-draw engine, built ON the existing cashflow grid + decumulation primitives -- NOT glue. Two genuinely new pieces: (a) per-month PLACEMENT of Social Security/pension/annuity income in the month each lands (today retirementIncomeMonthly() averages every source to one flat per-month figure and the cashflow grid adds it identically to all 12 months -- the cadence fields exist but are averaged away); (b) a per-month SAFE DRAW (withdrawalPlan() is annual-only today -- one flat yearly net withdrawal -- so 'safe draw $1,640 THIS month' does not yet exist as an object). Built atop the verified primitives (RateBand safe/moderate/high, withdrawalOrder, the lumpy cashflow grid).</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr"/>
-      <c r="G5" s="4" t="inlineStr"/>
-    </row>
-    <row r="6">
+      <c r="F5" s="4" t="n"/>
+      <c r="G5" s="4" t="n"/>
+    </row>
+    <row r="6" ht="112" customHeight="1">
       <c r="A6" s="6" t="inlineStr">
         <is>
           <t>Will-it-last / retirement confidence (single canonical home)</t>
@@ -874,10 +965,14 @@
           <t>Reuses the retirement Monte-Carlo engine (src/domain/retirement: simulate -&gt; p10/p50/p90 shown as best-to-worst, depletionAge, solveRetireAge) and RetirementCockpit.</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr"/>
-      <c r="G6" s="4" t="inlineStr"/>
-    </row>
-    <row r="7">
+      <c r="F6" s="4" t="n"/>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>Why retirement number resides in spend tab? What's the logical reason?</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="64" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
         <is>
           <t>Which-accounts-to-draw-from order</t>
@@ -903,10 +998,10 @@
           <t>Reuses decumulation withdrawalOrder + taxBucketSplit (verified built, RMD-aware from age 73).</t>
         </is>
       </c>
-      <c r="F7" s="4" t="inlineStr"/>
-      <c r="G7" s="4" t="inlineStr"/>
-    </row>
-    <row r="8">
+      <c r="F7" s="4" t="n"/>
+      <c r="G7" s="4" t="n"/>
+    </row>
+    <row r="8" ht="112" customHeight="1">
       <c r="A8" s="6" t="inlineStr">
         <is>
           <t>Chief-of-staff: Social Security claim-timing</t>
@@ -932,10 +1027,10 @@
           <t>Reuses retirement simulate (a guaranteed-income-start-age input already models Social Security starting at the claim age) + the will-it-last engine; a focused decision screen with a user-moved longevity slider wraps them.</t>
         </is>
       </c>
-      <c r="F8" s="4" t="inlineStr"/>
-      <c r="G8" s="4" t="inlineStr"/>
-    </row>
-    <row r="9">
+      <c r="F8" s="4" t="n"/>
+      <c r="G8" s="4" t="n"/>
+    </row>
+    <row r="9" ht="80" customHeight="1">
       <c r="A9" s="6" t="inlineStr">
         <is>
           <t>Chief-of-staff: retirement transition + required withdrawals</t>
@@ -961,10 +1056,10 @@
           <t>Reuses decumulation rmdAtAge / rmdDivisor / RMD_START_AGE (verified built); surfaced as reminders in 'What needs you'.</t>
         </is>
       </c>
-      <c r="F9" s="4" t="inlineStr"/>
-      <c r="G9" s="4" t="inlineStr"/>
-    </row>
-    <row r="10">
+      <c r="F9" s="4" t="n"/>
+      <c r="G9" s="4" t="n"/>
+    </row>
+    <row r="10" ht="80" customHeight="1">
       <c r="A10" s="6" t="inlineStr">
         <is>
           <t>'What needs you' -- quantified attention nudges</t>
@@ -990,10 +1085,10 @@
           <t>Reuses the insights engine (src/domain/insights: buildInsights, themes protect/grow/optimize) + InsightsScreen + contribution-room screen.</t>
         </is>
       </c>
-      <c r="F10" s="4" t="inlineStr"/>
-      <c r="G10" s="4" t="inlineStr"/>
-    </row>
-    <row r="11">
+      <c r="F10" s="4" t="n"/>
+      <c r="G10" s="4" t="n"/>
+    </row>
+    <row r="11" ht="80" customHeight="1">
       <c r="A11" s="6" t="inlineStr">
         <is>
           <t>The scenario engine (you run it, we never recommend)</t>
@@ -1019,8 +1114,8 @@
           <t>Reuses retirement simulate + projectNestEgg + solveRetireAge and the performance what-if; surfaced via the existing slider UI in RetirementCockpit and Performance.</t>
         </is>
       </c>
-      <c r="F11" s="4" t="inlineStr"/>
-      <c r="G11" s="4" t="inlineStr"/>
+      <c r="F11" s="4" t="n"/>
+      <c r="G11" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1033,17 +1128,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:E7"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="90" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="1" t="inlineStr"/>
+      <c r="A1" s="1" t="n"/>
       <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Detail</t>
@@ -1059,8 +1155,13 @@
           <t>💬 Comments</t>
         </is>
       </c>
-    </row>
-    <row r="2">
+      <c r="E1" s="9" t="inlineStr">
+        <is>
+          <t>💬 Claude response</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="96" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>NAV MODEL</t>
@@ -1071,10 +1172,10 @@
           <t>A persistent bottom tab bar (always reachable, large tap targets) with a single smart Home at the center. Home is the chief-of-staff dashboard and is the part that FLEXES between the two lenses: for the still-working it leads with Grow and Track, for the retired it leads with the Safe-to-spend paycheck. The other tabs are the same for both lenses -- only the hero emphasis and a couple of labels change. A 'Guide' tab is where the chief-of-staff big-decision walkthroughs live, so the heavy stuff has a calm home of its own and never clutters the daily view. Five tabs, all spelled out in full on screen (no cryptic truncations), keeps it glanceable on a phone.</t>
         </is>
       </c>
-      <c r="C2" s="4" t="inlineStr"/>
-      <c r="D2" s="4" t="inlineStr"/>
-    </row>
-    <row r="3">
+      <c r="C2" s="4" t="n"/>
+      <c r="D2" s="4" t="n"/>
+    </row>
+    <row r="3" ht="48" customHeight="1">
       <c r="A3" s="7" t="inlineStr">
         <is>
           <t>Home</t>
@@ -1085,10 +1186,10 @@
           <t>The chief-of-staff dashboard. Flexes by lens: hero = Grow and Track (working) or Safe-to-spend paycheck (retired); plus 'What needs you' and a will-it-last reassurance strip that links to its home in the Spend tab. The two-second glance.</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr"/>
-      <c r="D3" s="4" t="inlineStr"/>
-    </row>
-    <row r="4">
+      <c r="C3" s="4" t="n"/>
+      <c r="D3" s="4" t="n"/>
+    </row>
+    <row r="4" ht="32" customHeight="1">
       <c r="A4" s="7" t="inlineStr">
         <is>
           <t>Money</t>
@@ -1099,10 +1200,14 @@
           <t>Foundation: connected accounts, the whole-picture net worth, and income + spending by month including the dated big bills. The single true picture.</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr"/>
-      <c r="D4" s="4" t="inlineStr"/>
-    </row>
-    <row r="5">
+      <c r="C4" s="4" t="n"/>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>NW, Money, spending all in one screen is that too much?</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="32" customHeight="1">
       <c r="A5" s="7" t="inlineStr">
         <is>
           <t>Invest</t>
@@ -1113,10 +1218,10 @@
           <t>Grow and Track in depth: returns in percent and dollars, winners vs laggards, how you compare to the stock market, and the investment what-if scenarios. Emphasized for the still-working; present but lighter for the retired.</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr"/>
-      <c r="D5" s="4" t="inlineStr"/>
-    </row>
-    <row r="6">
+      <c r="C5" s="4" t="n"/>
+      <c r="D5" s="4" t="n"/>
+    </row>
+    <row r="6" ht="48" customHeight="1">
       <c r="A6" s="7" t="inlineStr">
         <is>
           <t>Spend</t>
@@ -1127,10 +1232,14 @@
           <t>Safe-to-spend in depth and the CANONICAL HOME of the will-it-last number: the month-by-month paycheck, which-accounts-to-draw-from order, and the odds your money lasts. Emphasized for the retired; for the still-working it shows a clearly-labeled PROJECTION of their future retirement paycheck.</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr"/>
-      <c r="D6" s="4" t="inlineStr"/>
-    </row>
-    <row r="7">
+      <c r="C6" s="4" t="n"/>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>Do not like the name</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="48" customHeight="1">
       <c r="A7" s="7" t="inlineStr">
         <is>
           <t>Guide</t>
@@ -1141,8 +1250,12 @@
           <t>The chief-of-staff big-decision walkthroughs: Social Security claim-timing, the retirement transition, required-withdrawal reminders -- each laying out the options in your dollars with deadlines and user-set assumptions. You decide.</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr"/>
-      <c r="D7" s="4" t="inlineStr"/>
+      <c r="C7" s="4" t="n"/>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>do not like the name</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1155,8 +1268,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:G7"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
@@ -1164,12 +1277,13 @@
     <col width="46" customWidth="1" min="4" max="4"/>
     <col width="11" customWidth="1" min="5" max="5"/>
     <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="60" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Screen</t>
+          <t>w</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -1197,8 +1311,13 @@
           <t>💬 Comments</t>
         </is>
       </c>
-    </row>
-    <row r="2" ht="340.2" customHeight="1">
+      <c r="G1" s="9" t="inlineStr">
+        <is>
+          <t>💬 Claude response</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="340.25" customHeight="1">
       <c r="A2" s="6" t="inlineStr">
         <is>
           <t>Home -- chief-of-staff dashboard (flexes by lens)</t>
@@ -1252,10 +1371,14 @@
 • Safe-to-spend labeled with the actual month to signal it changes month to month</t>
         </is>
       </c>
-      <c r="E2" s="4" t="inlineStr"/>
-      <c r="F2" s="4" t="inlineStr"/>
-    </row>
-    <row r="3" ht="352.8" customHeight="1">
+      <c r="E2" s="4" t="n"/>
+      <c r="F2" s="4" t="inlineStr">
+        <is>
+          <t>How you plan to capture the information?</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="352.75" customHeight="1">
       <c r="A3" s="6" t="inlineStr">
         <is>
           <t>Money -- whole-picture net worth + month-by-month, with dated big bills</t>
@@ -1309,10 +1432,10 @@
 • Hide-balances respected (masks all money); own/owe shown by label not color alone</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr"/>
-      <c r="F3" s="4" t="inlineStr"/>
-    </row>
-    <row r="4" ht="327.6" customHeight="1">
+      <c r="E3" s="4" t="n"/>
+      <c r="F3" s="4" t="n"/>
+    </row>
+    <row r="4" ht="327.5" customHeight="1">
       <c r="A4" s="6" t="inlineStr">
         <is>
           <t>Invest -- Grow &amp; Track with a what-if</t>
@@ -1365,8 +1488,12 @@
 • Reuses the Performance engine (attribution, market comparison, trend)</t>
         </is>
       </c>
-      <c r="E4" s="4" t="inlineStr"/>
-      <c r="F4" s="4" t="inlineStr"/>
+      <c r="E4" s="4" t="n"/>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>What's the level of details displayed and how?r</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="315" customHeight="1">
       <c r="A5" s="6" t="inlineStr">
@@ -1420,10 +1547,10 @@
 • Reuses decumulation withdrawalOrder + Monte-Carlo; the per-month income placement + per-month safe draw are the new engine</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr"/>
-      <c r="F5" s="4" t="inlineStr"/>
-    </row>
-    <row r="6" ht="340.2" customHeight="1">
+      <c r="E5" s="4" t="n"/>
+      <c r="F5" s="4" t="n"/>
+    </row>
+    <row r="6" ht="340.25" customHeight="1">
       <c r="A6" s="6" t="inlineStr">
         <is>
           <t>Guide -- Social Security claim-timing (chief of staff)</t>
@@ -1477,10 +1604,10 @@
 • Reuses retirement simulate with the guaranteed-income-start-age input + the will-it-last engine</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr"/>
-      <c r="F6" s="4" t="inlineStr"/>
-    </row>
-    <row r="7" ht="327.6" customHeight="1">
+      <c r="E6" s="4" t="n"/>
+      <c r="F6" s="4" t="n"/>
+    </row>
+    <row r="7" ht="327.5" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
         <is>
           <t>Connect accounts -- onboarding</t>
@@ -1533,8 +1660,8 @@
 • Reuses the secure read-only sync seam + existing manual account/holding editors</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr"/>
-      <c r="F7" s="4" t="inlineStr"/>
+      <c r="E7" s="4" t="n"/>
+      <c r="F7" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1547,13 +1674,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:E7"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="80" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -1577,8 +1705,13 @@
           <t>💬 Comments</t>
         </is>
       </c>
-    </row>
-    <row r="2">
+      <c r="E1" s="9" t="inlineStr">
+        <is>
+          <t>💬 Claude response</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="112" customHeight="1">
       <c r="A2" s="6" t="inlineStr">
         <is>
           <t>Still-working 55-65: 'How are my investments doing, and am I on track?'</t>
@@ -1592,10 +1725,14 @@
 4. Glances at the will-it-last strip on Home -&gt; 'Likely (84%)' -&gt; taps through to its home in Spend, reassured, closes app</t>
         </is>
       </c>
-      <c r="C2" s="4" t="inlineStr"/>
-      <c r="D2" s="4" t="inlineStr"/>
-    </row>
-    <row r="3">
+      <c r="C2" s="4" t="n"/>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>How about a scenario do I have enough to support my parents with $2500 per month, and still save for kids college, pay mortgage, and save for retirement? How will it impact by retirement paycheck or date?</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="96" customHeight="1">
       <c r="A3" s="6" t="inlineStr">
         <is>
           <t>Early-retired 65-70: 'How much can I safely spend this month?'</t>
@@ -1609,10 +1746,14 @@
 4. Sees will-it-last 'Likely 84%, range 71-95%' right there in its home -&gt; worries less, lives more</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr"/>
-      <c r="D3" s="4" t="inlineStr"/>
-    </row>
-    <row r="4">
+      <c r="C3" s="4" t="n"/>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>are month bars cashflows - showing inflow and outflow?</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="96" customHeight="1">
       <c r="A4" s="6" t="inlineStr">
         <is>
           <t>The big decision: when to claim Social Security (chief of staff)</t>
@@ -1626,10 +1767,10 @@
 4. Taps 'Remind me' for the September deadline and 'Compare' to run a what-if; makes the call themselves later</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr"/>
-      <c r="D4" s="4" t="inlineStr"/>
-    </row>
-    <row r="5">
+      <c r="C4" s="4" t="n"/>
+      <c r="D4" s="4" t="n"/>
+    </row>
+    <row r="5" ht="112" customHeight="1">
       <c r="A5" s="6" t="inlineStr">
         <is>
           <t>First run: connect accounts -&gt; see the whole picture</t>
@@ -1643,10 +1784,10 @@
 4. Continues -&gt; Money shows a single net-worth number with grouped own/owe; FinWise asks the stage question (still working vs retired) -&gt; Home picks the right lens</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr"/>
-      <c r="D5" s="4" t="inlineStr"/>
-    </row>
-    <row r="6">
+      <c r="C5" s="4" t="n"/>
+      <c r="D5" s="4" t="n"/>
+    </row>
+    <row r="6" ht="112" customHeight="1">
       <c r="A6" s="6" t="inlineStr">
         <is>
           <t>The transition: from Grow &amp; Track to Safe-to-spend</t>
@@ -1660,10 +1801,10 @@
 4. Same accounts, same engines, same net-worth truth -- only the face changed, so they never feel they outgrew the app</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr"/>
-      <c r="D6" s="4" t="inlineStr"/>
-    </row>
-    <row r="7">
+      <c r="C6" s="4" t="n"/>
+      <c r="D6" s="4" t="n"/>
+    </row>
+    <row r="7" ht="96" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
         <is>
           <t>Recurring nudge: 'What needs you' acted on by the user</t>
@@ -1677,8 +1818,8 @@
 4. User decides on their own and the nudge clears next time the picture updates -- a reason to keep coming back</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr"/>
-      <c r="D7" s="4" t="inlineStr"/>
+      <c r="C7" s="4" t="n"/>
+      <c r="D7" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
docs(FCC-core): answer ALL 13 review comments in the response column (was 3; +10 missed via truncated read)
Proactive 'what needs you' principle; 'can I afford home/college/parents' lives in Guide/
scenario layer (not Grow&Track); will-it-last placement fix; Money-tab summary-that-expands;
rename Spend+Guide (options+leans); Home capture cross-ref; Invest glance->drill; the multi-goal
trade-off scenario journey; month-bars-as-inflow/outflow. Decisions pending: Spend+Guide names.
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/FCC-core-highlevel-design-v1.0-2026-06-30.xlsx
+++ b/docs/FCC-core-55-70/FCC-core-highlevel-design-v1.0-2026-06-30.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="33600" windowHeight="19880" tabRatio="600" firstSheet="0" activeTab="4" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="33600" windowHeight="19880" tabRatio="600" firstSheet="0" activeTab="3" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Overview &amp; principles" sheetId="1" state="visible" r:id="rId1"/>
@@ -13,7 +13,7 @@
     <sheet name="Journeys" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -47,12 +47,14 @@
       <sz val="9"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <family val="2"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -81,7 +83,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001A1A18"/>
+        <fgColor rgb="FF1A1A18"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE2EFDA"/>
       </patternFill>
     </fill>
     <fill>
@@ -90,7 +97,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -115,6 +122,32 @@
     </border>
     <border>
       <left style="thin">
+        <color rgb="FFD9D9D9"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD9D9D9"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD9D9D9"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD9D9D9"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
         <color rgb="00D9D9D9"/>
       </left>
       <right style="thin">
@@ -131,7 +164,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -161,6 +194,15 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -582,15 +624,15 @@
           <t>Foundation layer only shows income, spending, and connected accounts as true picture. Three questions (1) Are these connected accounts checking, savings, investments, credit card or something different? (2) Via Plaid or anyother third party tool can the app actually pull real data without prompted by user daily? How will data be pulled, and at what frequency? (3) We said for this group - FinWise gives 36-to-65-year-olds one honest, engaging place to see their whole financial picture — led by how their investments and net worth are actually growing — and to explore the consequences of their big money choices for themselves. It matters because this group has the most money and the most at stake, yet no app shows them the whole truth clearly AND makes it something they actually want to open week to week. But that's not reflected in this overview or did I miss something?</t>
         </is>
       </c>
-      <c r="E2" s="10" t="inlineStr">
-        <is>
-          <t>(1) ACCOUNT TYPES: all of them — banking (checking/savings/cash management), INVESTMENTS (brokerage + retirement 401(k)/IRA — where the growth &amp; net-worth number lives), credit cards + loans; manual-add for what can't be linked (home value, pension, private assets).
-(2) PULL: yes, NO daily prompting. Connect each institution ONCE via an aggregator (Plaid is the standard); the connection persists. Data then auto-pulls — a DAILY refresh + a refresh each time the app opens. Read-only (we can never move money). ⚠ Privacy spike: Plaid routes data through its servers in transit, so 'never leaves your device' isn't literal — honest posture = read-only, on-device storage, encrypted, minimal retention, never sold (carries to the PRD/technical stage).
-(3) OBJECTIVE: you're right — it's a gap. The overview describes the shared core but doesn't foreground each group's objective/hook. FIX in v1.1: rewrite the overview to carry both groups' approved objectives (Grow &amp; Track / week-to-week for 55-65; safe-to-spend / worry-less for 65-70).</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="48" customHeight="1">
+      <c r="E2" s="13" t="inlineStr">
+        <is>
+          <t>(1) ACCOUNT TYPES: all of them — banking (checking/savings/cash mgmt), INVESTMENTS (brokerage + retirement 401(k)/IRA — where the growth &amp; net-worth number lives), credit cards + loans; manual-add for home value, pension, private assets.
+(2) PULL: yes, NO daily prompting. Connect each institution ONCE via an aggregator (Plaid is the standard); it persists, then auto-pulls daily + on each app open. Read-only. ⚠ Privacy spike: Plaid routes data through its servers in transit, so 'never leaves your device' isn't literal — honest posture = read-only, on-device storage, encrypted, minimal retention, never sold (carries to the PRD).
+(3) OBJECTIVE: you're right, it's a gap. v1.1 rewrites the overview to carry both groups' objectives (Grow &amp; Track / week-to-week for 55-65; safe-to-spend / worry-less for 65-70).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="170" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
         <is>
           <t>Principle 1</t>
@@ -605,6 +647,11 @@
       <c r="D3" s="4" t="inlineStr">
         <is>
           <t>Shall we also talk about - we surface right things at the right time - kind of what needs your attention.</t>
+        </is>
+      </c>
+      <c r="E3" s="13" t="inlineStr">
+        <is>
+          <t>YES — strong addition. v1.1 adds a PROACTIVE principle: we bring the right thing to your attention at the right time (a required withdrawal due, a Social Security claiming window closing, idle cash, a goal drifting off track) so you don't have to go looking. It's already half-present as the 'What needs you' element on Home; let's make it an explicit principle — it's the chief of staff being proactive.</t>
         </is>
       </c>
     </row>
@@ -745,7 +792,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -756,6 +803,7 @@
     <col width="11" customWidth="1" min="6" max="6"/>
     <col width="26" customWidth="1" min="7" max="7"/>
     <col width="60" customWidth="1" min="8" max="8"/>
+    <col width="25.1640625" customWidth="1" style="12" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -799,6 +847,11 @@
           <t>💬 Claude response</t>
         </is>
       </c>
+      <c r="I1" s="11" t="inlineStr">
+        <is>
+          <t>Comments</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="220" customHeight="1">
       <c r="A2" s="6" t="inlineStr">
@@ -832,10 +885,10 @@
           <t>Is it one time pull, daily, or initiated by user? What if user is hesitant to connects account in the beginning?</t>
         </is>
       </c>
-      <c r="H2" s="10" t="inlineStr">
+      <c r="H2" s="13" t="inlineStr">
         <is>
           <t>One-time connect -&gt; AUTOMATIC refresh (daily + on-open), NOT user-initiated each day. Read-only.
-HESITANCY (we don't force it): (a) START WITHOUT CONNECTING — manual/partial entry so they see the first 'aha' (net worth / a rough safe-to-spend) before linking anything; (b) PROGRESSIVE CONNECT — link the ONE account that unlocks the hero they care about (brokerage -&gt; Grow &amp; Track; checking + income -&gt; safe-to-spend), then invite more; (c) lead with read-only / on-device / never-sold as the trust + the reward. v1.1 adds a progressive-connect onboarding path.</t>
+HESITANCY (we don't force it): (a) START WITHOUT CONNECTING — manual/partial entry to see the first 'aha' (net worth / rough safe-to-spend) before linking; (b) PROGRESSIVE CONNECT — link the ONE account that unlocks the hero they care about (brokerage-&gt;Grow&amp;Track; checking+income-&gt;safe-to-spend), then invite more; (c) lead with read-only / on-device / never-sold as the trust + reward. v1.1 adds a progressive-connect onboarding path.</t>
         </is>
       </c>
     </row>
@@ -871,9 +924,14 @@
           <t>How all this information will be captured and at what frequency?</t>
         </is>
       </c>
-      <c r="H3" s="10" t="inlineStr">
-        <is>
-          <t>Mostly AUTOMATIC from the connected accounts on the same daily/on-open refresh (deposits -&gt; income, transactions -&gt; spending). DATED big bills (property tax in Nov, a pension lump in Dec) and anything not connected are MANUALLY added — that's what keeps safe-to-spend honest MONTH-BY-MONTH. So: auto from accounts + manual for dated lumpy items. v1.1 clarifies this on the row.</t>
+      <c r="H3" s="13" t="inlineStr">
+        <is>
+          <t>Mostly AUTOMATIC from the connected accounts on the same daily/on-open refresh (deposits-&gt;income, transactions-&gt;spending). DATED big bills (property tax in Nov, a pension lump in Dec) and anything not connected are MANUALLY added — that's what keeps safe-to-spend honest month-by-month. So: auto from accounts + manual for dated lumpy items.</t>
+        </is>
+      </c>
+      <c r="I3" s="12" t="inlineStr">
+        <is>
+          <t>What if person does not connect credit card accounts or has cash expenses?</t>
         </is>
       </c>
     </row>
@@ -904,9 +962,14 @@
         </is>
       </c>
       <c r="F4" s="4" t="n"/>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>Does this also answer questions about Can I efford an home, or kids college, or take care of parents as we laid out in strategy doc - "Your chief of staff for the BUILDING years — guides you through your investments, the home, the kids' college, and the run-up to retirement, so you build the life you're working toward. 'Grow' = watch your money grow (the hook); 'Track' = always know you're on track.</t>
+        </is>
+      </c>
+      <c r="H4" s="13" t="inlineStr">
+        <is>
+          <t>No — and good catch. Grow &amp; Track is only the INVESTMENT-growth view (the hook: returns, winners/laggards, vs market). 'Can I afford a home / kids' college / supporting parents' is a DIFFERENT capability: the chief-of-staff GUIDE + the scenario engine. v1.1 makes explicit that the Guide/scenario layer covers the 36-65 big decisions (afford-a-home, college, supporting parents, the run-up to retirement), not just Social Security timing. See the Journeys row on the multi-goal trade-off.</t>
         </is>
       </c>
     </row>
@@ -939,7 +1002,7 @@
       <c r="F5" s="4" t="n"/>
       <c r="G5" s="4" t="n"/>
     </row>
-    <row r="6" ht="112" customHeight="1">
+    <row r="6" ht="170" customHeight="1">
       <c r="A6" s="6" t="inlineStr">
         <is>
           <t>Will-it-last / retirement confidence (single canonical home)</t>
@@ -969,6 +1032,11 @@
       <c r="G6" s="4" t="inlineStr">
         <is>
           <t>Why retirement number resides in spend tab? What's the logical reason?</t>
+        </is>
+      </c>
+      <c r="H6" s="13" t="inlineStr">
+        <is>
+          <t>Fair challenge. The placement was retiree-centric: for the early-retired, 'will my money last' is the reassurance directly behind 'what can I safely spend,' so they sit together. BUT for the still-working 55-65 it's a TRACK/PLAN thing, not a Spend thing — so the placement is lopsided. v1.1: the will-it-last/retirement-confidence number gets a neutral home (the Home reassurance layer + a Plan/Track view); the Spend/paycheck tab shows it for retirees. (Ties to the Navigation comments.)</t>
         </is>
       </c>
     </row>
@@ -1189,7 +1257,7 @@
       <c r="C3" s="4" t="n"/>
       <c r="D3" s="4" t="n"/>
     </row>
-    <row r="4" ht="32" customHeight="1">
+    <row r="4" ht="170" customHeight="1">
       <c r="A4" s="7" t="inlineStr">
         <is>
           <t>Money</t>
@@ -1206,6 +1274,11 @@
           <t>NW, Money, spending all in one screen is that too much?</t>
         </is>
       </c>
+      <c r="E4" s="13" t="inlineStr">
+        <is>
+          <t>Agree it risks being crowded. Your expand/collapse instinct is the fix: a GLANCE summary (net worth + this-month cash) that EXPANDS into accounts/spending detail — not everything at once. Alternatively split Net Worth (whole picture / growth) from day-to-day Money/spending. v1.1: reconsider the Money tab as a summary-that-expands.</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="32" customHeight="1">
       <c r="A5" s="7" t="inlineStr">
@@ -1221,7 +1294,7 @@
       <c r="C5" s="4" t="n"/>
       <c r="D5" s="4" t="n"/>
     </row>
-    <row r="6" ht="48" customHeight="1">
+    <row r="6" ht="170" customHeight="1">
       <c r="A6" s="7" t="inlineStr">
         <is>
           <t>Spend</t>
@@ -1238,8 +1311,13 @@
           <t>Do not like the name</t>
         </is>
       </c>
-    </row>
-    <row r="7" ht="48" customHeight="1">
+      <c r="E6" s="13" t="inlineStr">
+        <is>
+          <t>Agree — 'Spend' sounds like we're nudging you to spend. Options: 'Paycheck' (retiree framing — your safe monthly paycheck), 'Cash flow' (neutral, cross-lens), 'Safe to spend', or 'Income'. My lean: 'Paycheck' for the retiree lens, 'Cash flow' as the shared name. Your call — I'll rename in v1.1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="170" customHeight="1">
       <c r="A7" s="7" t="inlineStr">
         <is>
           <t>Guide</t>
@@ -1254,6 +1332,11 @@
       <c r="D7" s="4" t="inlineStr">
         <is>
           <t>do not like the name</t>
+        </is>
+      </c>
+      <c r="E7" s="13" t="inlineStr">
+        <is>
+          <t>Agree. For the big-decisions / chief-of-staff tab: 'Plan', 'Decisions', 'Big moves', or 'Navigate'. My lean: 'Plan' (broad — holds the scenarios + the big decisions) or 'Decisions' (sharper). NOT 'Advisor' (we're deliberately not one). Your call — rename in v1.1.</t>
         </is>
       </c>
     </row>
@@ -1377,6 +1460,11 @@
           <t>How you plan to capture the information?</t>
         </is>
       </c>
+      <c r="G2" s="13" t="inlineStr">
+        <is>
+          <t>Same as the data-layer answer (Overview + Connect-accounts rows): Home DISPLAYS data captured automatically from your connected accounts (daily + on-open refresh) plus anything you manually added. Home is a display surface; capture happens via connect-once + manual — no separate capture here.</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="352.75" customHeight="1">
       <c r="A3" s="6" t="inlineStr">
@@ -1492,6 +1580,11 @@
       <c r="F4" s="4" t="inlineStr">
         <is>
           <t>What's the level of details displayed and how?r</t>
+        </is>
+      </c>
+      <c r="G4" s="13" t="inlineStr">
+        <is>
+          <t>Glance (top): total return %/$ for the period + how you're doing vs the market. Drill (tap): winners vs laggards, by account, and the what-if scenario. Principle = glanceable summary first, detail on tap (progressive disclosure). Exact layout is the next gate (detailed design); v1.1 notes the summary-&gt;drill structure.</t>
         </is>
       </c>
     </row>
@@ -1711,7 +1804,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="112" customHeight="1">
+    <row r="2" ht="170" customHeight="1">
       <c r="A2" s="6" t="inlineStr">
         <is>
           <t>Still-working 55-65: 'How are my investments doing, and am I on track?'</t>
@@ -1731,8 +1824,13 @@
           <t>How about a scenario do I have enough to support my parents with $2500 per month, and still save for kids college, pay mortgage, and save for retirement? How will it impact by retirement paycheck or date?</t>
         </is>
       </c>
-    </row>
-    <row r="3" ht="96" customHeight="1">
+      <c r="E2" s="13" t="inlineStr">
+        <is>
+          <t>YES — this is THE killer chief-of-staff capability for 36-65, exactly what the scenario engine is for. Journey: 'Can I support my parents at $2,500/mo AND keep saving for college, the mortgage, and retirement — what does it do to my retirement date/paycheck?' We show the trade-off in your real numbers (each goal funded or not + the hit to your retirement date/confidence); you decide. v1.1: add this MULTI-GOAL trade-off as a key journey + ensure the scenario engine handles multiple simultaneous goals, not one decision at a time.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="170" customHeight="1">
       <c r="A3" s="6" t="inlineStr">
         <is>
           <t>Early-retired 65-70: 'How much can I safely spend this month?'</t>
@@ -1752,6 +1850,11 @@
           <t>are month bars cashflows - showing inflow and outflow?</t>
         </is>
       </c>
+      <c r="E3" s="13" t="inlineStr">
+        <is>
+          <t>Good question — let's make them exactly that. The month bars show safe-to-spend by month AND its composition: guaranteed income in (Social Security + pension), the safe draw from savings, and the dated big bills out — so each bar reads as the real inflow/outflow that produces that month's number (Nov dip = property tax, Dec lift = pension lump). v1.1: clarify the month bars as inflow/outflow composition, like the onboarding cash-flow chart.</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="96" customHeight="1">
       <c r="A4" s="6" t="inlineStr">

</xml_diff>